<commit_message>
fix(04d): Include Elastic Net and Ridge in 8-method consensus
CRITICAL FIX:
- 04d_stability_consensus.py was only using 6 methods (Spearman, MI, ANOVA, RFECV, Lasso, RF)
- Elastic Net and Ridge were computed in 04c but NOT used in consensus
- Now uses all 8 methods: 3 filter + 1 wrapper + 4 embedded

METHODOLOGY CHANGES:
- Consensus intersection now requires agreement from all 8 methods
- Tighter consensus results in fewer but more robust features
- Base and nested variants now produce identical feature sets

FEATURE COUNTS (v1.1):
- H1: 9 features (was 10)
- H2: 9 features (unchanged)
- H3: 5 features (was 7)
- H4: 7 features (was 8)
- H5: 9 features (was 10)

PIPELINE RERUN: 04d -> 05 -> 05b -> 06 (both base and nested variants)

Updated addendum.tex claims to correctly describe 8-method consensus.
</commit_message>
<xml_diff>
--- a/results/04_feature_selection/04d_ALL_consensus.xlsx
+++ b/results/04_feature_selection/04d_ALL_consensus.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,20 +471,25 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Nested_Stability_Avg</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Baseline_ROC_AUC</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Consensus_ROC_AUC</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Retention_%</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Threshold_Met</t>
         </is>
@@ -500,7 +505,7 @@
         <v>40</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -508,21 +513,24 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>75</v>
+        <v>77.5</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6089432035781782</v>
+        <v>0.6387926515082863</v>
       </c>
       <c r="G2" t="n">
+        <v>0.2769115477721268</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.7715858062343247</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.7827777918629683</v>
-      </c>
       <c r="I2" t="n">
-        <v>101.4505173032233</v>
-      </c>
-      <c r="J2" t="inlineStr">
+        <v>0.7830138502042437</v>
+      </c>
+      <c r="J2" t="n">
+        <v>101.4811112228325</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -549,18 +557,21 @@
         <v>78.04878048780488</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5608411849797064</v>
+        <v>0.6064131946658647</v>
       </c>
       <c r="G3" t="n">
+        <v>0.295146051008736</v>
+      </c>
+      <c r="H3" t="n">
         <v>0.7092283022813564</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>0.6846025597459205</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>96.52781164313059</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -576,7 +587,7 @@
         <v>42</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -584,21 +595,24 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>83.33333333333334</v>
+        <v>88.09523809523809</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5363286331617156</v>
+        <v>0.4692218250748227</v>
       </c>
       <c r="G4" t="n">
+        <v>0.4193757988861722</v>
+      </c>
+      <c r="H4" t="n">
         <v>0.7317904491106442</v>
       </c>
-      <c r="H4" t="n">
-        <v>0.7436214385423241</v>
-      </c>
       <c r="I4" t="n">
-        <v>101.6167182075222</v>
-      </c>
-      <c r="J4" t="inlineStr">
+        <v>0.7371297104138026</v>
+      </c>
+      <c r="J4" t="n">
+        <v>100.7296161503129</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -614,7 +628,7 @@
         <v>43</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -622,21 +636,24 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>81.3953488372093</v>
+        <v>83.72093023255813</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5431621920034563</v>
+        <v>0.5876632501947429</v>
       </c>
       <c r="G5" t="n">
+        <v>0.322242066632012</v>
+      </c>
+      <c r="H5" t="n">
         <v>0.7584511382732912</v>
       </c>
-      <c r="H5" t="n">
-        <v>0.740204074741885</v>
-      </c>
       <c r="I5" t="n">
-        <v>97.5941675593041</v>
-      </c>
-      <c r="J5" t="inlineStr">
+        <v>0.7423180768872754</v>
+      </c>
+      <c r="J5" t="n">
+        <v>97.87289377365234</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -652,7 +669,7 @@
         <v>41</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -660,21 +677,24 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>75.60975609756098</v>
+        <v>78.04878048780488</v>
       </c>
       <c r="F6" t="n">
-        <v>0.580675491793581</v>
+        <v>0.6050546722159541</v>
       </c>
       <c r="G6" t="n">
+        <v>0.3803651501032307</v>
+      </c>
+      <c r="H6" t="n">
         <v>0.8468093876883849</v>
       </c>
-      <c r="H6" t="n">
-        <v>0.8380082807867801</v>
-      </c>
       <c r="I6" t="n">
-        <v>98.96067438203183</v>
-      </c>
-      <c r="J6" t="inlineStr">
+        <v>0.8384060741259433</v>
+      </c>
+      <c r="J6" t="n">
+        <v>99.00764992870698</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -691,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,19 +739,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.8125</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -746,28 +766,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7441860465116279</v>
+        <v>0.8604651162790697</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.6774193548387096</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="D4" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -778,11 +798,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.8125</v>
       </c>
       <c r="D5" t="n">
         <v>26</v>
@@ -791,181 +811,181 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.5757575757575758</v>
+        <v>0.7</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6904761904761905</v>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6774193548387096</v>
       </c>
       <c r="D8" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.5581395348837209</v>
+        <v>0.6511627906976745</v>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.525</v>
+        <v>0.6511627906976745</v>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5135135135135135</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.6190476190476191</v>
       </c>
       <c r="D12" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.6</v>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.4</v>
+        <v>0.5952380952380952</v>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.5813953488372093</v>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -976,13 +996,247 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="D16" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5581395348837209</v>
+      </c>
+      <c r="D17" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="D18" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="D19" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.5121951219512195</v>
+      </c>
+      <c r="D20" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5116279069767442</v>
+      </c>
+      <c r="D21" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.4871794871794872</v>
+      </c>
+      <c r="D22" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="D23" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>RFECV</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.4523809523809524</v>
+      </c>
+      <c r="D24" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D25" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.4117647058823529</v>
+      </c>
+      <c r="D26" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D27" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.3902439024390244</v>
+      </c>
+      <c r="D28" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D29" t="n">
         <v>12</v>
       </c>
     </row>
@@ -997,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1043,37 +1297,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7575757575757576</v>
+        <v>0.84375</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -1084,47 +1338,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.675</v>
+        <v>0.8125</v>
       </c>
       <c r="D5" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.5853658536585366</v>
+        <v>0.7575757575757576</v>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.5853658536585366</v>
+        <v>0.7058823529411765</v>
       </c>
       <c r="D7" t="n">
         <v>24</v>
@@ -1133,61 +1387,61 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.5853658536585366</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="D8" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="D10" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1196,28 +1450,28 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5483870967741935</v>
+        <v>0.6216216216216216</v>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.5384615384615384</v>
+        <v>0.6</v>
       </c>
       <c r="D12" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -1228,67 +1482,301 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.4375</v>
+        <v>0.6</v>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.4375</v>
+        <v>0.5853658536585366</v>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.4375</v>
+        <v>0.5853658536585366</v>
       </c>
       <c r="D15" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5853658536585366</v>
+      </c>
+      <c r="D16" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5789473684210527</v>
+      </c>
+      <c r="D17" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.5789473684210527</v>
+      </c>
+      <c r="D18" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="D19" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="D20" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>RFECV</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5517241379310345</v>
+      </c>
+      <c r="D21" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.5483870967741935</v>
+      </c>
+      <c r="D22" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.5405405405405406</v>
+      </c>
+      <c r="D23" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D26" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D27" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D28" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>Random_Forest</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C29" t="n">
         <v>0.325</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D29" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1303,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1390,24 +1878,54 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1, A2, A3, A5, A6, A9, A13, A15, A17, A21...</t>
+          <t>A1, A3, A5, A6, A9, A12, A13, A15, A20, A21...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>40</v>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>A1, A2, A3, A5, A6, A9, A12, A13, A15, A17...</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A12, A28, A60, A15, A45, A2, A41, A36, A3, A21...</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>40</v>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>A1, A2, A3, A5, A6, A9, A12, A13, A15, A17...</t>
         </is>
@@ -1424,7 +1942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1515,20 +2033,50 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A2, A3, A5, A6, A9, A12, A15, A17, A20, A21...</t>
+          <t>A2, A3, A5, A6, A9, A12, A15, A20, A21, A24...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>40</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A1, A2, A3, A5, A6, A9, A12, A15, A17, A20...</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>29</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A2, A21, A62, A6, A20, A31, A60, A56, A29, A41...</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Random_Forest</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" t="n">
         <v>41</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>A1, A2, A3, A5, A6, A9, A12, A15, A17, A20...</t>
         </is>
@@ -1545,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1632,24 +2180,54 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A2, A3, A6, A9, A11, A13, A15, A17, A20, A21...</t>
+          <t>A13, A15, A20, A21, A24, A26, A34, A35, A36, A38...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>18</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A13, A15, A20, A21, A24, A25, A26, A34, A35, A36...</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>30</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A58, A17, A64, A34, A53, A15, A41, A2, A11, A3...</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Random_Forest</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" t="n">
         <v>42</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>A2, A3, A5, A6, A9, A11, A12, A13, A15, A17...</t>
         </is>
@@ -1666,7 +2244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1753,24 +2331,54 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1, A5, A6, A9, A12, A13, A15, A17, A20, A21...</t>
+          <t>A1, A2, A3, A5, A6, A9, A12, A13, A15, A17...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>39</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A1, A2, A3, A5, A6, A9, A13, A15, A17, A20...</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>29</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A24, A5, A3, A6, A59, A64, A41, A35, A30, A53...</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Random_Forest</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" t="n">
         <v>38</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>A2, A3, A5, A6, A9, A12, A13, A17, A20, A21...</t>
         </is>
@@ -1787,7 +2395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1878,20 +2486,50 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1, A3, A5, A20, A21, A24, A25, A26, A27, A29...</t>
+          <t>A1, A3, A5, A12, A20, A21, A24, A25, A26, A27...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>28</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A1, A3, A20, A21, A24, A25, A26, A27, A29, A34...</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>27</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A55, A37, A27, A12, A42, A58, A44, A57, A30, A40...</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Random_Forest</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" t="n">
         <v>36</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>A3, A5, A6, A9, A12, A15, A17, A20, A21, A24...</t>
         </is>
@@ -1908,7 +2546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1936,7 +2574,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1945,46 +2583,46 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7575757575757576</v>
+        <v>0.9</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.9</v>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -1995,32 +2633,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.725</v>
+        <v>0.7575757575757576</v>
       </c>
       <c r="D5" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.725</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -2031,14 +2669,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6842105263157895</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="D7" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -2049,38 +2687,38 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6774193548387096</v>
+        <v>0.725</v>
       </c>
       <c r="D8" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6410256410256411</v>
+        <v>0.725</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2089,64 +2727,64 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.575</v>
+        <v>0.725</v>
       </c>
       <c r="D10" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5675675675675675</v>
+        <v>0.725</v>
       </c>
       <c r="D11" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.7</v>
       </c>
       <c r="D12" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.4375</v>
+        <v>0.7</v>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -2157,50 +2795,284 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.4375</v>
+        <v>0.6774193548387096</v>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="D15" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D16" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D17" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>RFECV</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.6071428571428571</v>
+      </c>
+      <c r="D18" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D19" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="D20" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="D21" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>Random_Forest</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C22" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="D22" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.5128205128205128</v>
+      </c>
+      <c r="D23" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D24" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D25" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="D26" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
         <v>0.425</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D27" t="n">
         <v>17</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="D28" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.3947368421052632</v>
+      </c>
+      <c r="D29" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2214,7 +3086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2242,7 +3114,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2251,64 +3123,64 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.926829268292683</v>
+        <v>0.975609756097561</v>
       </c>
       <c r="D2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.75</v>
+        <v>0.926829268292683</v>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.9024390243902439</v>
       </c>
       <c r="D4" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.6333333333333333</v>
+        <v>0.7631578947368421</v>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
@@ -2319,38 +3191,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.5862068965517241</v>
+        <v>0.725</v>
       </c>
       <c r="D7" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2359,64 +3231,64 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.5609756097560976</v>
+        <v>0.7073170731707317</v>
       </c>
       <c r="D8" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.5609756097560976</v>
+        <v>0.65</v>
       </c>
       <c r="D9" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.525</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.525</v>
+        <v>0.6333333333333333</v>
       </c>
       <c r="D11" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -2427,14 +3299,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.4814814814814815</v>
+        <v>0.625</v>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -2445,11 +3317,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.4473684210526316</v>
+        <v>0.5862068965517241</v>
       </c>
       <c r="D13" t="n">
         <v>17</v>
@@ -2458,54 +3330,288 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.4333333333333333</v>
+        <v>0.5862068965517241</v>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.4146341463414634</v>
+        <v>0.575</v>
       </c>
       <c r="D15" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="D16" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="D17" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Mutual_Info</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.5641025641025641</v>
+      </c>
+      <c r="D18" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.5609756097560976</v>
+      </c>
+      <c r="D19" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.5609756097560976</v>
+      </c>
+      <c r="D20" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5609756097560976</v>
+      </c>
+      <c r="D21" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="D22" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.4857142857142857</v>
+      </c>
+      <c r="D23" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>RFECV</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C24" t="n">
+        <v>0.4814814814814815</v>
+      </c>
+      <c r="D24" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.4473684210526316</v>
+      </c>
+      <c r="D25" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.4333333333333333</v>
+      </c>
+      <c r="D26" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="D27" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.4146341463414634</v>
+      </c>
+      <c r="D28" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D29" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2520,7 +3626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2548,37 +3654,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="D2" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7931034482758621</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="D3" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -2620,7 +3726,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2629,16 +3735,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6904761904761905</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2647,10 +3753,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.6904761904761905</v>
       </c>
       <c r="D7" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -2674,144 +3780,378 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6153846153846154</v>
+        <v>0.6190476190476191</v>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5384615384615384</v>
+        <v>0.5945945945945946</v>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5384615384615384</v>
+        <v>0.5483870967741935</v>
       </c>
       <c r="D11" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.2580645161290323</v>
+        <v>0.5135135135135135</v>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.5135135135135135</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="D16" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Random_Forest</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.3809523809523809</v>
+      </c>
+      <c r="D17" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>RFECV</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="D20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="D21" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.2941176470588235</v>
+      </c>
+      <c r="D22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.2941176470588235</v>
+      </c>
+      <c r="D23" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Ridge_L2</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.2903225806451613</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lasso_L1</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="D25" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.2580645161290323</v>
+      </c>
+      <c r="D26" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.2413793103448276</v>
+      </c>
+      <c r="D27" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.2413793103448276</v>
+      </c>
+      <c r="D28" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RFECV</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>Random_Forest</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C29" t="n">
         <v>0.2380952380952381</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D29" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(04d): Use 8-method consensus with proper base/nested variant handling
CRITICAL FIX: 04d_stability_consensus.py was only using 6 methods for consensus
(excluding Elastic Net and Ridge computed in 04c). This has been fixed to use
all 8 methods: 3 filter + 1 wrapper + 4 embedded.

Additionally fixed --variant flag to properly switch between:
- BASE: Uses non-nested embedded selections (direct selected_features)
- NESTED: Uses nested CV embedded results (majority voting over 5 folds)

Results now show meaningful differences between base and nested:
- H1: 10→9 features (A35 dropped - unstable in nested Lasso)
- H2: 9→9 features (no change)
- H3: 6→5 features (A49 dropped), winner changed RF→ExtraTrees
- H4: 8→7 features (A12 dropped)
- H5: 10→9 features (A30 dropped)

The nested approach is more conservative because it requires features to be
selected in >50% of CV folds, filtering out features that were selected due
to overfitting to specific train/test splits.
</commit_message>
<xml_diff>
--- a/results/04_feature_selection/04d_ALL_consensus.xlsx
+++ b/results/04_feature_selection/04d_ALL_consensus.xlsx
@@ -505,7 +505,7 @@
         <v>40</v>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>77.5</v>
+        <v>75</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6387926515082863</v>
+        <v>0.6505563576087073</v>
       </c>
       <c r="G2" t="n">
         <v>0.2769115477721268</v>
@@ -525,10 +525,10 @@
         <v>0.7715858062343247</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7830138502042437</v>
+        <v>0.7827777918629683</v>
       </c>
       <c r="J2" t="n">
-        <v>101.4811112228325</v>
+        <v>101.4505173032233</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -557,7 +557,7 @@
         <v>78.04878048780488</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6064131946658647</v>
+        <v>0.6089314305598287</v>
       </c>
       <c r="G3" t="n">
         <v>0.295146051008736</v>
@@ -587,7 +587,7 @@
         <v>42</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -595,10 +595,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>88.09523809523809</v>
+        <v>85.71428571428572</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4692218250748227</v>
+        <v>0.5432321035921207</v>
       </c>
       <c r="G4" t="n">
         <v>0.4193757988861722</v>
@@ -607,10 +607,10 @@
         <v>0.7317904491106442</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7371297104138026</v>
+        <v>0.7416451769600094</v>
       </c>
       <c r="J4" t="n">
-        <v>100.7296161503129</v>
+        <v>101.3466598069628</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -628,7 +628,7 @@
         <v>43</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -636,10 +636,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>83.72093023255813</v>
+        <v>81.3953488372093</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5876632501947429</v>
+        <v>0.5852666247103888</v>
       </c>
       <c r="G5" t="n">
         <v>0.322242066632012</v>
@@ -648,10 +648,10 @@
         <v>0.7584511382732912</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7423180768872754</v>
+        <v>0.740204074741885</v>
       </c>
       <c r="J5" t="n">
-        <v>97.87289377365234</v>
+        <v>97.5941675593041</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
         <v>41</v>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -677,10 +677,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>78.04878048780488</v>
+        <v>75.60975609756098</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6050546722159541</v>
+        <v>0.6278525961324934</v>
       </c>
       <c r="G6" t="n">
         <v>0.3803651501032307</v>
@@ -689,10 +689,10 @@
         <v>0.8468093876883849</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8384060741259433</v>
+        <v>0.8380082807867801</v>
       </c>
       <c r="J6" t="n">
-        <v>99.00764992870698</v>
+        <v>98.96067438203183</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -748,16 +748,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9024390243902439</v>
       </c>
       <c r="D2" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -766,70 +766,70 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.8604651162790697</v>
+        <v>0.8372093023255814</v>
       </c>
       <c r="D3" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8125</v>
       </c>
       <c r="D4" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8125</v>
+        <v>0.8108108108108109</v>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.7</v>
+        <v>0.7441860465116279</v>
       </c>
       <c r="D6" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -838,10 +838,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6904761904761905</v>
+        <v>0.7317073170731707</v>
       </c>
       <c r="D7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
@@ -870,32 +870,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6511627906976745</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="D9" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.6511627906976745</v>
+        <v>0.6333333333333333</v>
       </c>
       <c r="D10" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -906,14 +906,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.6279069767441861</v>
       </c>
       <c r="D11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -928,82 +928,82 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.6279069767441861</v>
       </c>
       <c r="D12" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.6</v>
+        <v>0.6190476190476191</v>
       </c>
       <c r="D13" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.5952380952380952</v>
+        <v>0.5757575757575758</v>
       </c>
       <c r="D14" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.5813953488372093</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="D15" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.5757575757575758</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="D16" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17">
@@ -1036,10 +1036,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.5526315789473685</v>
       </c>
       <c r="D18" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19">
@@ -1063,106 +1063,106 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5135135135135135</v>
       </c>
       <c r="D20" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.5116279069767442</v>
+        <v>0.5128205128205128</v>
       </c>
       <c r="D21" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.4871794871794872</v>
+        <v>0.4883720930232558</v>
       </c>
       <c r="D22" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.4857142857142857</v>
+        <v>0.4634146341463415</v>
       </c>
       <c r="D23" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.4324324324324325</v>
       </c>
       <c r="D24" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.45</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D25" t="n">
         <v>18</v>
@@ -1306,10 +1306,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.84375</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="D3" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -1324,10 +1324,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8787878787878788</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -1342,10 +1342,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8125</v>
+        <v>0.8484848484848485</v>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -1387,43 +1387,43 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6470588235294118</v>
+        <v>0.7</v>
       </c>
       <c r="D8" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.6857142857142857</v>
       </c>
       <c r="D9" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1432,34 +1432,34 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.6296296296296297</v>
+        <v>0.6857142857142857</v>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6216216216216216</v>
+        <v>0.675</v>
       </c>
       <c r="D11" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1468,43 +1468,43 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="D12" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.6</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="D13" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.5853658536585366</v>
+        <v>0.6486486486486487</v>
       </c>
       <c r="D14" t="n">
         <v>24</v>
@@ -1531,7 +1531,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1549,19 +1549,19 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.5853658536585366</v>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
@@ -1585,25 +1585,25 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.575</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="D19" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1612,16 +1612,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="D20" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1630,46 +1630,46 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.5641025641025641</v>
       </c>
       <c r="D21" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.5483870967741935</v>
+        <v>0.5526315789473685</v>
       </c>
       <c r="D22" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.5405405405405406</v>
+        <v>0.5483870967741935</v>
       </c>
       <c r="D23" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24">
@@ -1680,20 +1680,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.5</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="D24" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1702,16 +1702,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.5</v>
+        <v>0.53125</v>
       </c>
       <c r="D25" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1729,7 +1729,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1878,11 +1878,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1, A3, A5, A6, A9, A12, A13, A15, A20, A21...</t>
+          <t>A1, A2, A3, A5, A6, A9, A13, A15, A17, A21...</t>
         </is>
       </c>
     </row>
@@ -1908,11 +1908,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A12, A28, A60, A15, A45, A2, A41, A36, A3, A21...</t>
+          <t>A6, A5, A59, A55, A57, A15, A28, A33, A2, A41...</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A2, A3, A5, A6, A9, A12, A15, A20, A21, A24...</t>
+          <t>A2, A3, A5, A6, A9, A12, A15, A17, A20, A21...</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2059,11 +2059,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A2, A21, A62, A6, A20, A31, A60, A56, A29, A41...</t>
+          <t>A21, A5, A31, A20, A2, A57, A6, A60, A15, A55...</t>
         </is>
       </c>
     </row>
@@ -2180,11 +2180,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A13, A15, A20, A21, A24, A26, A34, A35, A36, A38...</t>
+          <t>A2, A3, A6, A9, A11, A13, A15, A17, A20, A21...</t>
         </is>
       </c>
     </row>
@@ -2195,11 +2195,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A13, A15, A20, A21, A24, A25, A26, A34, A35, A36...</t>
+          <t>A3, A9, A13, A15, A20, A21, A24, A25, A26, A27...</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A58, A17, A64, A34, A53, A15, A41, A2, A11, A3...</t>
+          <t>A29, A56, A17, A64, A33, A27, A58, A12, A55, A41...</t>
         </is>
       </c>
     </row>
@@ -2331,11 +2331,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1, A2, A3, A5, A6, A9, A12, A13, A15, A17...</t>
+          <t>A1, A5, A6, A9, A12, A13, A15, A17, A20, A21...</t>
         </is>
       </c>
     </row>
@@ -2346,11 +2346,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A1, A2, A3, A5, A6, A9, A13, A15, A17, A20...</t>
+          <t>A1, A2, A3, A5, A6, A9, A12, A13, A15, A17...</t>
         </is>
       </c>
     </row>
@@ -2361,11 +2361,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A24, A5, A3, A6, A59, A64, A41, A35, A30, A53...</t>
+          <t>A59, A30, A20, A27, A31, A64, A12, A5, A6, A44...</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1, A3, A5, A12, A20, A21, A24, A25, A26, A27...</t>
+          <t>A1, A3, A5, A20, A21, A24, A25, A26, A27, A29...</t>
         </is>
       </c>
     </row>
@@ -2497,11 +2497,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A1, A3, A20, A21, A24, A25, A26, A27, A29, A34...</t>
+          <t>A1, A3, A5, A15, A17, A20, A21, A24, A25, A26...</t>
         </is>
       </c>
     </row>
@@ -2512,11 +2512,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A55, A37, A27, A12, A42, A58, A44, A57, A30, A40...</t>
+          <t>A33, A56, A17, A5, A37, A30, A27, A55, A57, A59...</t>
         </is>
       </c>
     </row>
@@ -2597,14 +2597,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="D3" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -2615,14 +2615,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="D4" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -2646,25 +2646,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.7567567567567568</v>
       </c>
       <c r="D6" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2673,16 +2673,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.75</v>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2691,10 +2691,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.725</v>
+        <v>0.75</v>
       </c>
       <c r="D8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -2705,14 +2705,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.725</v>
+        <v>0.7352941176470589</v>
       </c>
       <c r="D9" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -2723,25 +2723,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.725</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="D10" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -2754,25 +2754,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Mutual_Info</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Elastic_Net</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Ridge_L2</t>
-        </is>
-      </c>
       <c r="C12" t="n">
-        <v>0.7</v>
+        <v>0.725</v>
       </c>
       <c r="D12" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2781,46 +2781,46 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.7</v>
+        <v>0.725</v>
       </c>
       <c r="D13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.6774193548387096</v>
+        <v>0.725</v>
       </c>
       <c r="D14" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.6842105263157895</v>
       </c>
       <c r="D15" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -2831,20 +2831,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.625</v>
+        <v>0.6774193548387096</v>
       </c>
       <c r="D16" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.625</v>
+        <v>0.6410256410256411</v>
       </c>
       <c r="D17" t="n">
         <v>25</v>
@@ -2862,7 +2862,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2871,28 +2871,28 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.6071428571428571</v>
+        <v>0.6388888888888888</v>
       </c>
       <c r="D18" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.6</v>
+        <v>0.575</v>
       </c>
       <c r="D19" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20">
@@ -2903,14 +2903,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.59375</v>
+        <v>0.575</v>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21">
@@ -2921,32 +2921,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.575</v>
+        <v>0.5675675675675675</v>
       </c>
       <c r="D21" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.575</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="D22" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23">
@@ -2957,38 +2957,38 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.5128205128205128</v>
+        <v>0.5588235294117647</v>
       </c>
       <c r="D23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.4375</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="D24" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3006,7 +3006,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3015,28 +3015,28 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.4375</v>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>ANOVA_F</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>RFECV</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Elastic_Net</t>
-        </is>
-      </c>
       <c r="C27" t="n">
-        <v>0.425</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D27" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3065,14 +3065,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.3947368421052632</v>
+        <v>0.425</v>
       </c>
       <c r="D29" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -3123,10 +3123,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.975609756097561</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -3159,10 +3159,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9024390243902439</v>
+        <v>0.926829268292683</v>
       </c>
       <c r="D4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7631578947368421</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="D5" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -3204,37 +3204,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.725</v>
+        <v>0.7317073170731707</v>
       </c>
       <c r="D7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Elastic_Net</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Ridge_L2</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Random_Forest</t>
-        </is>
-      </c>
       <c r="C8" t="n">
-        <v>0.7073170731707317</v>
+        <v>0.7317073170731707</v>
       </c>
       <c r="D8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.65</v>
+        <v>0.6341463414634146</v>
       </c>
       <c r="D9" t="n">
         <v>26</v>
@@ -3303,7 +3303,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.625</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="D12" t="n">
         <v>20</v>
@@ -3312,37 +3312,37 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.5862068965517241</v>
+        <v>0.6</v>
       </c>
       <c r="D13" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.5862068965517241</v>
+        <v>0.6</v>
       </c>
       <c r="D14" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -3353,50 +3353,50 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.575</v>
+        <v>0.5862068965517241</v>
       </c>
       <c r="D15" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.575</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="D16" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.5609756097560976</v>
       </c>
       <c r="D17" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18">
@@ -3407,25 +3407,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.5641025641025641</v>
+        <v>0.5609756097560976</v>
       </c>
       <c r="D18" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -3438,12 +3438,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -3461,20 +3461,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.5609756097560976</v>
+        <v>0.525</v>
       </c>
       <c r="D21" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3501,10 +3501,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.4857142857142857</v>
+        <v>0.5142857142857142</v>
       </c>
       <c r="D23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24">
@@ -3569,11 +3569,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.425</v>
+        <v>0.4146341463414634</v>
       </c>
       <c r="D27" t="n">
         <v>17</v>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3654,19 +3654,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7931034482758621</v>
+        <v>0.8529411764705882</v>
       </c>
       <c r="D2" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -3677,14 +3677,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -3695,25 +3695,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7741935483870968</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Mutual_Info</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -3726,61 +3726,61 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.7741935483870968</v>
       </c>
       <c r="D6" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>Elastic_Net</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6904761904761905</v>
+        <v>0.7352941176470589</v>
       </c>
       <c r="D7" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.7297297297297297</v>
       </c>
       <c r="D8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3789,10 +3789,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="D9" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
@@ -3803,14 +3803,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5945945945945946</v>
+        <v>0.6904761904761905</v>
       </c>
       <c r="D10" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11">
@@ -3821,128 +3821,128 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5483870967741935</v>
+        <v>0.6904761904761905</v>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.6190476190476191</v>
       </c>
       <c r="D12" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Random_Forest</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.5135135135135135</v>
+        <v>0.6190476190476191</v>
       </c>
       <c r="D13" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.5135135135135135</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.5526315789473685</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Elastic_Net</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Random_Forest</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="D16" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Lasso_L1</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Random_Forest</t>
-        </is>
-      </c>
       <c r="C17" t="n">
-        <v>0.3809523809523809</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="D17" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RFECV</t>
+          <t>Mutual_Info</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3951,10 +3951,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4871794871794872</v>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
@@ -3965,14 +3965,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.3125</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="D19" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
@@ -3983,20 +3983,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.3125</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="D20" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4005,16 +4005,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.3055555555555556</v>
+        <v>0.4102564102564102</v>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4023,16 +4023,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.4102564102564102</v>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.3448275862068966</v>
       </c>
       <c r="D23" t="n">
         <v>10</v>
@@ -4055,32 +4055,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ridge_L2</t>
+          <t>Lasso_L1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mutual_Info</t>
+          <t>RFECV</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Lasso_L1</t>
+          <t>Ridge_L2</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="D25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
@@ -4104,7 +4104,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ANOVA_F</t>
+          <t>Spearman</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4122,7 +4122,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Spearman</t>
+          <t>ANOVA_F</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">

</xml_diff>